<commit_message>
Private Markets Modelling and Commitment Planning
</commit_message>
<xml_diff>
--- a/epsilon-phi-core/src/Scripts/Case Studies/Private Assets/Simple Analysis.xlsx
+++ b/epsilon-phi-core/src/Scripts/Case Studies/Private Assets/Simple Analysis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/Repositories/Python/epsilon-phi/epsilon-phi-core/src/Scripts/Case Studies/Private Assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francisbarker/repo/epsilon-psi/epsilon-phi-core/src/Scripts/Case Studies/Private Assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568A64C4-A75D-C34F-A87D-BCE002C51FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025FF7AB-84D8-1848-A867-64F8C505D765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19800" yWindow="4780" windowWidth="20320" windowHeight="19040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13280" yWindow="500" windowWidth="20320" windowHeight="19040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolios" sheetId="2" r:id="rId1"/>
@@ -1011,6 +1011,7 @@
     <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1050,7 +1051,6 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="header_style" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -4968,232 +4968,232 @@
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="49"/>
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="114" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="113"/>
-      <c r="D1" s="113" t="s">
+      <c r="C1" s="114"/>
+      <c r="D1" s="114" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="113"/>
-      <c r="F1" s="113" t="s">
+      <c r="E1" s="114"/>
+      <c r="F1" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="113"/>
-      <c r="H1" s="113" t="s">
+      <c r="G1" s="114"/>
+      <c r="H1" s="114" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="114"/>
+      <c r="I1" s="115"/>
     </row>
     <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="115">
+      <c r="B2" s="116">
         <v>0.745</v>
       </c>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115" t="s">
+      <c r="C2" s="116"/>
+      <c r="D2" s="116" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115">
+      <c r="E2" s="116"/>
+      <c r="F2" s="116">
         <v>0.36</v>
       </c>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115">
+      <c r="G2" s="116"/>
+      <c r="H2" s="116">
         <v>0.15</v>
       </c>
-      <c r="I2" s="115"/>
+      <c r="I2" s="116"/>
     </row>
     <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="108">
+      <c r="B3" s="109">
         <v>0.02</v>
       </c>
-      <c r="C3" s="108"/>
-      <c r="D3" s="108">
+      <c r="C3" s="109"/>
+      <c r="D3" s="109">
         <v>0.03</v>
       </c>
-      <c r="E3" s="108"/>
-      <c r="F3" s="108">
+      <c r="E3" s="109"/>
+      <c r="F3" s="109">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G3" s="108"/>
-      <c r="H3" s="108">
+      <c r="G3" s="109"/>
+      <c r="H3" s="109">
         <v>5.5E-2</v>
       </c>
-      <c r="I3" s="108"/>
+      <c r="I3" s="109"/>
     </row>
     <row r="4" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="108">
+      <c r="B4" s="109">
         <v>0.14000000000000001</v>
       </c>
-      <c r="C4" s="108"/>
-      <c r="D4" s="108">
+      <c r="C4" s="109"/>
+      <c r="D4" s="109">
         <v>0.22500000000000001</v>
       </c>
-      <c r="E4" s="108"/>
-      <c r="F4" s="108">
+      <c r="E4" s="109"/>
+      <c r="F4" s="109">
         <v>0.35499999999999998</v>
       </c>
-      <c r="G4" s="108"/>
-      <c r="H4" s="108">
+      <c r="G4" s="109"/>
+      <c r="H4" s="109">
         <v>0.505</v>
       </c>
-      <c r="I4" s="108"/>
+      <c r="I4" s="109"/>
     </row>
     <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="108">
+      <c r="B5" s="109">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C5" s="108"/>
-      <c r="D5" s="108">
+      <c r="C5" s="109"/>
+      <c r="D5" s="109">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E5" s="108"/>
-      <c r="F5" s="108">
+      <c r="E5" s="109"/>
+      <c r="F5" s="109">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="G5" s="108"/>
-      <c r="H5" s="108">
+      <c r="G5" s="109"/>
+      <c r="H5" s="109">
         <v>0.03</v>
       </c>
-      <c r="I5" s="108"/>
+      <c r="I5" s="109"/>
     </row>
     <row r="6" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="108">
+      <c r="B6" s="109">
         <v>0.04</v>
       </c>
-      <c r="C6" s="108"/>
-      <c r="D6" s="108">
+      <c r="C6" s="109"/>
+      <c r="D6" s="109">
         <v>5.5E-2</v>
       </c>
-      <c r="E6" s="108"/>
-      <c r="F6" s="108">
+      <c r="E6" s="109"/>
+      <c r="F6" s="109">
         <v>0.12</v>
       </c>
-      <c r="G6" s="108"/>
-      <c r="H6" s="108">
+      <c r="G6" s="109"/>
+      <c r="H6" s="109">
         <v>0.185</v>
       </c>
-      <c r="I6" s="108"/>
+      <c r="I6" s="109"/>
     </row>
     <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="109">
+      <c r="B7" s="110">
         <v>0.04</v>
       </c>
-      <c r="C7" s="109"/>
-      <c r="D7" s="109">
+      <c r="C7" s="110"/>
+      <c r="D7" s="110">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E7" s="109"/>
-      <c r="F7" s="109">
+      <c r="E7" s="110"/>
+      <c r="F7" s="110">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G7" s="109"/>
-      <c r="H7" s="109">
+      <c r="G7" s="110"/>
+      <c r="H7" s="110">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="I7" s="109"/>
+      <c r="I7" s="110"/>
     </row>
     <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="110">
+      <c r="B8" s="111">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="C8" s="110"/>
-      <c r="D8" s="110">
+      <c r="C8" s="111"/>
+      <c r="D8" s="111">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E8" s="110"/>
-      <c r="F8" s="110">
+      <c r="E8" s="111"/>
+      <c r="F8" s="111">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G8" s="110"/>
-      <c r="H8" s="110">
+      <c r="G8" s="111"/>
+      <c r="H8" s="111">
         <v>7.5999999999999998E-2</v>
       </c>
-      <c r="I8" s="110"/>
+      <c r="I8" s="111"/>
     </row>
     <row r="9" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="111">
+      <c r="B9" s="112">
         <v>0.6</v>
       </c>
-      <c r="C9" s="111"/>
-      <c r="D9" s="111">
+      <c r="C9" s="112"/>
+      <c r="D9" s="112">
         <v>0.59</v>
       </c>
-      <c r="E9" s="111"/>
-      <c r="F9" s="111">
+      <c r="E9" s="112"/>
+      <c r="F9" s="112">
         <v>0.53</v>
       </c>
-      <c r="G9" s="111"/>
-      <c r="H9" s="111">
+      <c r="G9" s="112"/>
+      <c r="H9" s="112">
         <v>0.49</v>
       </c>
-      <c r="I9" s="111"/>
+      <c r="I9" s="112"/>
     </row>
     <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="108">
+      <c r="B10" s="109">
         <v>3.1E-2</v>
       </c>
-      <c r="C10" s="108"/>
-      <c r="D10" s="108">
+      <c r="C10" s="109"/>
+      <c r="D10" s="109">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="E10" s="108"/>
-      <c r="F10" s="108">
+      <c r="E10" s="109"/>
+      <c r="F10" s="109">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="G10" s="108"/>
-      <c r="H10" s="108">
+      <c r="G10" s="109"/>
+      <c r="H10" s="109">
         <v>0.10299999999999999</v>
       </c>
-      <c r="I10" s="108"/>
+      <c r="I10" s="109"/>
     </row>
     <row r="11" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="112" t="s">
+      <c r="B11" s="113" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="112"/>
-      <c r="D11" s="112" t="s">
+      <c r="C11" s="113"/>
+      <c r="D11" s="113" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="112"/>
-      <c r="F11" s="112" t="s">
+      <c r="E11" s="113"/>
+      <c r="F11" s="113" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="112"/>
-      <c r="H11" s="112" t="s">
+      <c r="G11" s="113"/>
+      <c r="H11" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="I11" s="112"/>
+      <c r="I11" s="113"/>
     </row>
     <row r="12" spans="1:9" s="8" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="55" t="s">
@@ -5486,64 +5486,64 @@
       <c r="A23" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="106">
+      <c r="B23" s="107">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="C23" s="106"/>
-      <c r="D23" s="106">
+      <c r="C23" s="107"/>
+      <c r="D23" s="107">
         <v>3.7999999999999999E-2</v>
       </c>
-      <c r="E23" s="106"/>
-      <c r="F23" s="106">
+      <c r="E23" s="107"/>
+      <c r="F23" s="107">
         <v>6.3E-2</v>
       </c>
-      <c r="G23" s="106"/>
-      <c r="H23" s="106">
+      <c r="G23" s="107"/>
+      <c r="H23" s="107">
         <v>8.8999999999999996E-2</v>
       </c>
-      <c r="I23" s="106"/>
+      <c r="I23" s="107"/>
     </row>
     <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="106">
+      <c r="B24" s="107">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C24" s="106"/>
-      <c r="D24" s="106">
+      <c r="C24" s="107"/>
+      <c r="D24" s="107">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="E24" s="106"/>
-      <c r="F24" s="106">
+      <c r="E24" s="107"/>
+      <c r="F24" s="107">
         <v>0.16200000000000001</v>
       </c>
-      <c r="G24" s="106"/>
-      <c r="H24" s="106">
+      <c r="G24" s="107"/>
+      <c r="H24" s="107">
         <v>0.24299999999999999</v>
       </c>
-      <c r="I24" s="106"/>
+      <c r="I24" s="107"/>
     </row>
     <row r="25" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="107">
+      <c r="B25" s="108">
         <v>0</v>
       </c>
-      <c r="C25" s="107"/>
-      <c r="D25" s="107">
+      <c r="C25" s="108"/>
+      <c r="D25" s="108">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="E25" s="107"/>
-      <c r="F25" s="107">
+      <c r="E25" s="108"/>
+      <c r="F25" s="108">
         <v>0.14899999999999999</v>
       </c>
-      <c r="G25" s="107"/>
-      <c r="H25" s="107">
+      <c r="G25" s="108"/>
+      <c r="H25" s="108">
         <v>0.253</v>
       </c>
-      <c r="I25" s="107"/>
+      <c r="I25" s="108"/>
     </row>
     <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="63" t="s">
@@ -5562,64 +5562,64 @@
       <c r="A27" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="106">
+      <c r="B27" s="107">
         <v>0.23799999999999999</v>
       </c>
-      <c r="C27" s="106"/>
-      <c r="D27" s="106">
+      <c r="C27" s="107"/>
+      <c r="D27" s="107">
         <v>0.27900000000000003</v>
       </c>
-      <c r="E27" s="106"/>
-      <c r="F27" s="106">
+      <c r="E27" s="107"/>
+      <c r="F27" s="107">
         <v>0.314</v>
       </c>
-      <c r="G27" s="106"/>
-      <c r="H27" s="106">
+      <c r="G27" s="107"/>
+      <c r="H27" s="107">
         <v>0.33700000000000002</v>
       </c>
-      <c r="I27" s="106"/>
+      <c r="I27" s="107"/>
     </row>
     <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="106">
+      <c r="B28" s="107">
         <v>0.04</v>
       </c>
-      <c r="C28" s="106"/>
-      <c r="D28" s="106">
+      <c r="C28" s="107"/>
+      <c r="D28" s="107">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="E28" s="106"/>
-      <c r="F28" s="106">
+      <c r="E28" s="107"/>
+      <c r="F28" s="107">
         <v>0.14299999999999999</v>
       </c>
-      <c r="G28" s="106"/>
-      <c r="H28" s="106">
+      <c r="G28" s="107"/>
+      <c r="H28" s="107">
         <v>0.187</v>
       </c>
-      <c r="I28" s="106"/>
+      <c r="I28" s="107"/>
     </row>
     <row r="29" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="B29" s="106">
+      <c r="B29" s="107">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C29" s="106"/>
-      <c r="D29" s="106">
+      <c r="C29" s="107"/>
+      <c r="D29" s="107">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="E29" s="106"/>
-      <c r="F29" s="106">
+      <c r="E29" s="107"/>
+      <c r="F29" s="107">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G29" s="106"/>
-      <c r="H29" s="106">
+      <c r="G29" s="107"/>
+      <c r="H29" s="107">
         <v>0.108</v>
       </c>
-      <c r="I29" s="106"/>
+      <c r="I29" s="107"/>
     </row>
     <row r="30" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="55" t="s">
@@ -6676,16 +6676,16 @@
   <sheetData>
     <row r="1" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="15"/>
-      <c r="B1" s="118" t="s">
+      <c r="B1" s="119" t="s">
         <v>95</v>
       </c>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
+      <c r="C1" s="119"/>
+      <c r="D1" s="119"/>
+      <c r="E1" s="119"/>
+      <c r="F1" s="119"/>
+      <c r="G1" s="119"/>
+      <c r="H1" s="119"/>
+      <c r="I1" s="119"/>
       <c r="J1" s="17"/>
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
@@ -6693,13 +6693,13 @@
     </row>
     <row r="2" spans="1:16" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="18"/>
-      <c r="B2" s="116" t="s">
+      <c r="B2" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="116"/>
-      <c r="D2" s="117"/>
-      <c r="E2" s="117"/>
-      <c r="F2" s="117"/>
+      <c r="C2" s="117"/>
+      <c r="D2" s="118"/>
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
       <c r="G2" s="20" t="s">
         <v>30</v>
       </c>
@@ -8098,7 +8098,7 @@
       <c r="D11">
         <v>0.13581920590229701</v>
       </c>
-      <c r="E11" s="119">
+      <c r="E11" s="106">
         <v>4.2297713801359103E-6</v>
       </c>
     </row>

</xml_diff>